<commit_message>
Correciones y boton de descargar
</commit_message>
<xml_diff>
--- a/notebooks/Outputs Excel/Horario_Cursos_MMDD.xlsx
+++ b/notebooks/Outputs Excel/Horario_Cursos_MMDD.xlsx
@@ -5719,7 +5719,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -6404,7 +6404,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -7089,7 +7089,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -7774,7 +7774,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -8459,7 +8459,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -9144,7 +9144,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -9829,7 +9829,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -10510,7 +10510,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -11191,7 +11191,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -11892,7 +11892,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -13557,7 +13557,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -14258,7 +14258,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -14959,7 +14959,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -15705,7 +15705,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -16451,7 +16451,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -17197,7 +17197,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -17943,7 +17943,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -18844,7 +18844,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -19745,7 +19745,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -20646,7 +20646,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -21543,7 +21543,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -21903,7 +21903,7 @@
     <row r="2">
       <c r="B2" s="29" t="inlineStr">
         <is>
-          <t>INFORME DE CUMPLIMIENTO Y FACTIBILIDAD — AÑO ESCOLAR 2026</t>
+          <t>INFORME DE CUMPLIMIENTO Y FACTIBILIDAD — AÑO ESCOLAR 2027</t>
         </is>
       </c>
     </row>
@@ -22174,7 +22174,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -22562,7 +22562,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -22954,7 +22954,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -23631,7 +23631,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -24308,7 +24308,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>
@@ -24993,7 +24993,7 @@
     </row>
     <row r="6">
       <c r="B6" s="12" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="7" ht="5.25" customHeight="1"/>

</xml_diff>